<commit_message>
Fix July 2 review data - correct 13 branches with wrong monthly/daily counts
</commit_message>
<xml_diff>
--- a/data/reviews.xlsx
+++ b/data/reviews.xlsx
@@ -23,11 +23,11 @@
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0_);[Red]&quot;(₹&quot;#,##0\)"/>
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="166" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="169" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="170" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="168" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="169" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="170" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="171" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -707,7 +707,7 @@
     <xf numFmtId="0" fontId="21" fillId="10" borderId="9" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1">
@@ -737,7 +737,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1">
@@ -746,7 +746,7 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1">
@@ -758,7 +758,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="7" applyAlignment="1">
@@ -774,7 +774,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -841,7 +841,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -849,6 +849,9 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1629,7 +1632,7 @@
         <v>28</v>
       </c>
       <c r="AG3" s="3" t="n"/>
-      <c r="AH3" s="24" t="n">
+      <c r="AH3" s="27" t="n">
         <v>46203</v>
       </c>
     </row>
@@ -1645,17 +1648,18 @@
         </is>
       </c>
       <c r="C4" s="15" t="n">
-        <v>7064</v>
+        <v>7087</v>
       </c>
       <c r="D4" s="3">
         <f>SUM(E4:AH4)</f>
         <v/>
       </c>
-      <c r="E4" s="3" t="n">
-        <v>20</v>
+      <c r="E4" s="3">
+        <f>SUM(E4:AH4)</f>
+        <v/>
       </c>
       <c r="F4" s="3" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>15</v>
@@ -1754,17 +1758,18 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>6386</v>
+        <v>6404</v>
       </c>
       <c r="D5" s="3">
         <f>SUM(E5:AH5)</f>
         <v/>
       </c>
-      <c r="E5" s="3" t="n">
-        <v>4</v>
+      <c r="E5" s="3">
+        <f>SUM(E5:AH5)</f>
+        <v/>
       </c>
       <c r="F5" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>7</v>
@@ -1863,17 +1868,18 @@
         </is>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="D6" s="3">
         <f>SUM(E6:AH6)</f>
         <v/>
       </c>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
+      <c r="E6" s="3">
+        <f>SUM(E6:AH6)</f>
+        <v/>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>3</v>
@@ -1972,14 +1978,15 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="D7" s="3">
         <f>SUM(E7:AH7)</f>
         <v/>
       </c>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
+      <c r="E7" s="3">
+        <f>SUM(E7:AH7)</f>
+        <v/>
       </c>
       <c r="F7" s="3" t="n">
         <v>1</v>
@@ -2081,17 +2088,18 @@
         </is>
       </c>
       <c r="C8" s="15" t="n">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="D8" s="3">
         <f>SUM(E8:AH8)</f>
         <v/>
       </c>
-      <c r="E8" s="3" t="n">
-        <v>2</v>
+      <c r="E8" s="3">
+        <f>SUM(E8:AH8)</f>
+        <v/>
       </c>
       <c r="F8" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>3</v>
@@ -2190,17 +2198,18 @@
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>2009</v>
+        <v>2017</v>
       </c>
       <c r="D9" s="3">
         <f>SUM(E9:AH9)</f>
         <v/>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>2</v>
+      <c r="E9" s="3">
+        <f>SUM(E9:AH9)</f>
+        <v/>
       </c>
       <c r="F9" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>3</v>
@@ -2299,17 +2308,18 @@
         </is>
       </c>
       <c r="C10" s="15" t="n">
-        <v>4292</v>
+        <v>4279</v>
       </c>
       <c r="D10" s="3">
         <f>SUM(E10:AH10)</f>
         <v/>
       </c>
-      <c r="E10" s="3" t="n">
-        <v>11</v>
+      <c r="E10" s="3">
+        <f>SUM(E10:AH10)</f>
+        <v/>
       </c>
       <c r="F10" s="3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>9</v>
@@ -2408,17 +2418,18 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>1170</v>
+        <v>1172</v>
       </c>
       <c r="D11" s="3">
         <f>SUM(E11:AH11)</f>
         <v/>
       </c>
-      <c r="E11" s="3" t="n">
-        <v>5</v>
+      <c r="E11" s="3">
+        <f>SUM(E11:AH11)</f>
+        <v/>
       </c>
       <c r="F11" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>1</v>
@@ -2517,14 +2528,15 @@
         </is>
       </c>
       <c r="C12" s="15" t="n">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="D12" s="3">
         <f>SUM(E12:AH12)</f>
         <v/>
       </c>
-      <c r="E12" s="3" t="n">
-        <v>3</v>
+      <c r="E12" s="3">
+        <f>SUM(E12:AH12)</f>
+        <v/>
       </c>
       <c r="F12" s="3" t="n">
         <v>2</v>
@@ -2626,17 +2638,18 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="D13" s="3">
         <f>SUM(E13:AH13)</f>
         <v/>
       </c>
-      <c r="E13" s="3" t="n">
-        <v>4</v>
+      <c r="E13" s="3">
+        <f>SUM(E13:AH13)</f>
+        <v/>
       </c>
       <c r="F13" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>1</v>
@@ -2732,21 +2745,22 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>4.7★</t>
+          <t>4.8★</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>3142</v>
+        <v>3153</v>
       </c>
       <c r="D14" s="3">
         <f>SUM(E14:AH14)</f>
         <v/>
       </c>
-      <c r="E14" s="3" t="n">
-        <v>1</v>
+      <c r="E14" s="3">
+        <f>SUM(E14:AH14)</f>
+        <v/>
       </c>
       <c r="F14" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>2</v>
@@ -2845,17 +2859,18 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>1131</v>
+        <v>1135</v>
       </c>
       <c r="D15" s="3">
         <f>SUM(E15:AH15)</f>
         <v/>
       </c>
-      <c r="E15" s="3" t="n">
-        <v>6</v>
+      <c r="E15" s="3">
+        <f>SUM(E15:AH15)</f>
+        <v/>
       </c>
       <c r="F15" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>9</v>
@@ -2954,17 +2969,18 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>1118</v>
+        <v>1124</v>
       </c>
       <c r="D16" s="3">
         <f>SUM(E16:AH16)</f>
         <v/>
       </c>
-      <c r="E16" s="3" t="n">
-        <v>8</v>
+      <c r="E16" s="3">
+        <f>SUM(E16:AH16)</f>
+        <v/>
       </c>
       <c r="F16" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>2</v>
@@ -3063,17 +3079,18 @@
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D17" s="3">
         <f>SUM(E17:AH17)</f>
         <v/>
       </c>
-      <c r="E17" s="3" t="n">
-        <v>0</v>
+      <c r="E17" s="3">
+        <f>SUM(E17:AH17)</f>
+        <v/>
       </c>
       <c r="F17" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>1</v>
@@ -3172,17 +3189,18 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D18" s="3">
         <f>SUM(E18:AH18)</f>
         <v/>
       </c>
-      <c r="E18" s="3" t="n">
-        <v>8</v>
+      <c r="E18" s="3">
+        <f>SUM(E18:AH18)</f>
+        <v/>
       </c>
       <c r="F18" s="3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>5</v>
@@ -3281,17 +3299,18 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D19" s="3">
         <f>SUM(E19:AH19)</f>
         <v/>
       </c>
-      <c r="E19" s="3" t="n">
-        <v>2</v>
+      <c r="E19" s="3">
+        <f>SUM(E19:AH19)</f>
+        <v/>
       </c>
       <c r="F19" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>3</v>
@@ -3390,17 +3409,18 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="D20" s="3">
         <f>SUM(E20:AH20)</f>
         <v/>
       </c>
-      <c r="E20" s="3" t="n">
-        <v>6</v>
+      <c r="E20" s="3">
+        <f>SUM(E20:AH20)</f>
+        <v/>
       </c>
       <c r="F20" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>1</v>
@@ -3499,17 +3519,18 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>2452</v>
+        <v>2475</v>
       </c>
       <c r="D21" s="3">
         <f>SUM(E21:AH21)</f>
         <v/>
       </c>
-      <c r="E21" s="3" t="n">
-        <v>1</v>
+      <c r="E21" s="3">
+        <f>SUM(E21:AH21)</f>
+        <v/>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>3</v>
@@ -3608,17 +3629,18 @@
         </is>
       </c>
       <c r="C22" s="15" t="n">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="D22" s="3">
         <f>SUM(E22:AH22)</f>
         <v/>
       </c>
-      <c r="E22" s="3" t="n">
-        <v>16</v>
+      <c r="E22" s="3">
+        <f>SUM(E22:AH22)</f>
+        <v/>
       </c>
       <c r="F22" s="3" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>6</v>
@@ -3717,17 +3739,18 @@
         </is>
       </c>
       <c r="C23" s="15" t="n">
-        <v>1152</v>
+        <v>1148</v>
       </c>
       <c r="D23" s="3">
         <f>SUM(E23:AH23)</f>
         <v/>
       </c>
-      <c r="E23" s="3" t="n">
-        <v>9</v>
+      <c r="E23" s="3">
+        <f>SUM(E23:AH23)</f>
+        <v/>
       </c>
       <c r="F23" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>10</v>
@@ -3826,17 +3849,18 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="D24" s="3">
         <f>SUM(E24:AH24)</f>
         <v/>
       </c>
-      <c r="E24" s="3" t="n">
-        <v>4</v>
+      <c r="E24" s="3">
+        <f>SUM(E24:AH24)</f>
+        <v/>
       </c>
       <c r="F24" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>4</v>
@@ -3935,17 +3959,18 @@
         </is>
       </c>
       <c r="C25" s="15" t="n">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="D25" s="3">
         <f>SUM(E25:AH25)</f>
         <v/>
       </c>
-      <c r="E25" s="3" t="n">
-        <v>2</v>
+      <c r="E25" s="3">
+        <f>SUM(E25:AH25)</f>
+        <v/>
       </c>
       <c r="F25" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>0</v>
@@ -4044,17 +4069,18 @@
         </is>
       </c>
       <c r="C26" s="15" t="n">
-        <v>971</v>
+        <v>978</v>
       </c>
       <c r="D26" s="3">
         <f>SUM(E26:AH26)</f>
         <v/>
       </c>
-      <c r="E26" s="3" t="n">
-        <v>6</v>
+      <c r="E26" s="3">
+        <f>SUM(E26:AH26)</f>
+        <v/>
       </c>
       <c r="F26" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>3</v>
@@ -4153,17 +4179,18 @@
         </is>
       </c>
       <c r="C27" s="15" t="n">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="D27" s="3">
         <f>SUM(E27:AH27)</f>
         <v/>
       </c>
-      <c r="E27" s="3" t="n">
-        <v>1</v>
+      <c r="E27" s="3">
+        <f>SUM(E27:AH27)</f>
+        <v/>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>3</v>
@@ -4262,17 +4289,18 @@
         </is>
       </c>
       <c r="C28" s="15" t="n">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="D28" s="3">
         <f>SUM(E28:AH28)</f>
         <v/>
       </c>
-      <c r="E28" s="3" t="n">
-        <v>3</v>
+      <c r="E28" s="3">
+        <f>SUM(E28:AH28)</f>
+        <v/>
       </c>
       <c r="F28" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>1</v>
@@ -4371,17 +4399,18 @@
         </is>
       </c>
       <c r="C29" s="15" t="n">
-        <v>6137</v>
+        <v>6154</v>
       </c>
       <c r="D29" s="3">
         <f>SUM(E29:AH29)</f>
         <v/>
       </c>
-      <c r="E29" s="3" t="n">
-        <v>3</v>
+      <c r="E29" s="3">
+        <f>SUM(E29:AH29)</f>
+        <v/>
       </c>
       <c r="F29" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>4</v>
@@ -4486,11 +4515,12 @@
         <f>SUM(E30:AH30)</f>
         <v/>
       </c>
-      <c r="E30" s="3" t="n">
-        <v>5</v>
+      <c r="E30" s="3">
+        <f>SUM(E30:AH30)</f>
+        <v/>
       </c>
       <c r="F30" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>3</v>
@@ -4589,17 +4619,18 @@
         </is>
       </c>
       <c r="C31" s="15" t="n">
-        <v>2249</v>
+        <v>2255</v>
       </c>
       <c r="D31" s="3">
         <f>SUM(E31:AH31)</f>
         <v/>
       </c>
-      <c r="E31" s="3" t="n">
-        <v>11</v>
+      <c r="E31" s="3">
+        <f>SUM(E31:AH31)</f>
+        <v/>
       </c>
       <c r="F31" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>10</v>
@@ -4698,17 +4729,18 @@
         </is>
       </c>
       <c r="C32" s="15" t="n">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="D32" s="3">
         <f>SUM(E32:AH32)</f>
         <v/>
       </c>
-      <c r="E32" s="3" t="n">
-        <v>4</v>
+      <c r="E32" s="3">
+        <f>SUM(E32:AH32)</f>
+        <v/>
       </c>
       <c r="F32" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>2</v>
@@ -4807,17 +4839,18 @@
         </is>
       </c>
       <c r="C33" s="15" t="n">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="D33" s="3">
         <f>SUM(E33:AH33)</f>
         <v/>
       </c>
-      <c r="E33" s="3" t="n">
-        <v>4</v>
+      <c r="E33" s="3">
+        <f>SUM(E33:AH33)</f>
+        <v/>
       </c>
       <c r="F33" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>1</v>
@@ -4916,17 +4949,18 @@
         </is>
       </c>
       <c r="C34" s="15" t="n">
-        <v>2096</v>
+        <v>2090</v>
       </c>
       <c r="D34" s="3">
         <f>SUM(E34:AH34)</f>
         <v/>
       </c>
-      <c r="E34" s="3" t="n">
-        <v>4</v>
+      <c r="E34" s="3">
+        <f>SUM(E34:AH34)</f>
+        <v/>
       </c>
       <c r="F34" s="3" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>5</v>
@@ -5025,17 +5059,18 @@
         </is>
       </c>
       <c r="C35" s="15" t="n">
-        <v>2124</v>
+        <v>2128</v>
       </c>
       <c r="D35" s="3">
         <f>SUM(E35:AH35)</f>
         <v/>
       </c>
-      <c r="E35" s="3" t="n">
-        <v>1</v>
+      <c r="E35" s="3">
+        <f>SUM(E35:AH35)</f>
+        <v/>
       </c>
       <c r="F35" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>1</v>
@@ -5134,17 +5169,18 @@
         </is>
       </c>
       <c r="C36" s="15" t="n">
-        <v>1728</v>
+        <v>1708</v>
       </c>
       <c r="D36" s="3">
         <f>SUM(E36:AH36)</f>
         <v/>
       </c>
-      <c r="E36" s="3" t="n">
-        <v>1</v>
+      <c r="E36" s="3">
+        <f>SUM(E36:AH36)</f>
+        <v/>
       </c>
       <c r="F36" s="3" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>10</v>
@@ -5243,14 +5279,15 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="D37" s="3">
         <f>SUM(E37:AH37)</f>
         <v/>
       </c>
-      <c r="E37" s="3" t="n">
-        <v>6</v>
+      <c r="E37" s="3">
+        <f>SUM(E37:AH37)</f>
+        <v/>
       </c>
       <c r="F37" s="3" t="n">
         <v>2</v>
@@ -5352,14 +5389,15 @@
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="D38" s="3">
         <f>SUM(E38:AH38)</f>
         <v/>
       </c>
-      <c r="E38" s="3" t="n">
-        <v>7</v>
+      <c r="E38" s="3">
+        <f>SUM(E38:AH38)</f>
+        <v/>
       </c>
       <c r="F38" s="3" t="n">
         <v>1</v>
@@ -5461,17 +5499,18 @@
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>1213</v>
+        <v>1217</v>
       </c>
       <c r="D39" s="3">
         <f>SUM(E39:AH39)</f>
         <v/>
       </c>
-      <c r="E39" s="3" t="n">
-        <v>7</v>
+      <c r="E39" s="3">
+        <f>SUM(E39:AH39)</f>
+        <v/>
       </c>
       <c r="F39" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G39" s="3" t="n">
         <v>5</v>
@@ -5654,7 +5693,7 @@
         <v>3949</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>173</v>
+        <v>19</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>31</v>
@@ -5678,14 +5717,14 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>4.7★</t>
+          <t>4.8★</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3142</v>
+        <v>3153</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>192</v>
+        <v>25</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>26</v>
@@ -5711,10 +5750,10 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>6137</v>
+        <v>6154</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>176</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>23</v>
@@ -5740,10 +5779,10 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2452</v>
+        <v>2475</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>243</v>
+        <v>21</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>21</v>
@@ -5769,10 +5808,10 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>7064</v>
+        <v>7087</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>528</v>
+        <v>44</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>16</v>
@@ -5798,10 +5837,10 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>126</v>
+        <v>6</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>16</v>
@@ -5827,10 +5866,10 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>12</v>
@@ -5856,10 +5895,10 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>12</v>
@@ -5885,10 +5924,10 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1170</v>
+        <v>1172</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>11</v>
@@ -5914,10 +5953,10 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>107</v>
+        <v>4</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>11</v>
@@ -5943,10 +5982,10 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>4292</v>
+        <v>4279</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>351</v>
+        <v>17</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>10</v>
@@ -5972,10 +6011,10 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>121</v>
+        <v>4</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>10</v>
@@ -6001,10 +6040,10 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>6386</v>
+        <v>6404</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>243</v>
+        <v>12</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>8</v>
@@ -6030,10 +6069,10 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2009</v>
+        <v>2017</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>8</v>
@@ -6059,10 +6098,10 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>94</v>
+        <v>4</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>7</v>
@@ -6088,10 +6127,10 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>7</v>
@@ -6117,10 +6156,10 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2249</v>
+        <v>2255</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>164</v>
+        <v>4</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>7</v>
@@ -6146,10 +6185,10 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1111</v>
+        <v>1108</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>6</v>
@@ -6175,10 +6214,10 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>6</v>
@@ -6204,10 +6243,10 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2397</v>
+        <v>2400</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>186</v>
+        <v>9</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>6</v>
@@ -6233,10 +6272,10 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>1152</v>
+        <v>1148</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>118</v>
+        <v>7</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>6</v>
@@ -6262,10 +6301,10 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>103</v>
+        <v>5</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>6</v>
@@ -6291,10 +6330,10 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>6</v>
@@ -6320,10 +6359,10 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>1213</v>
+        <v>1217</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>74</v>
+        <v>5</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>6</v>
@@ -6349,10 +6388,10 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>5</v>
@@ -6378,10 +6417,10 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>971</v>
+        <v>978</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>5</v>
@@ -6407,10 +6446,10 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1728</v>
+        <v>1708</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>172</v>
+        <v>4</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>5</v>
@@ -6436,10 +6475,10 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>4</v>
@@ -6465,10 +6504,10 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>89</v>
+        <v>8</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>3</v>
@@ -6494,10 +6533,10 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>90</v>
+        <v>3</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>2</v>
@@ -6523,10 +6562,10 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>1131</v>
+        <v>1135</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>119</v>
+        <v>8</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>2</v>
@@ -6552,10 +6591,10 @@
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>2</v>
@@ -6581,10 +6620,10 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>2096</v>
+        <v>2090</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>165</v>
+        <v>12</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>2</v>
@@ -6610,10 +6649,10 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>2124</v>
+        <v>2128</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>2</v>
@@ -6639,10 +6678,10 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>1118</v>
+        <v>1124</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>1</v>
@@ -6668,10 +6707,10 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>1</v>
@@ -6707,17 +6746,11 @@
         </is>
       </c>
       <c r="B41" s="3">
-        <f>VALUE(SUBSTITUTE(B4,"★",""))</f>
-        <v/>
-      </c>
-      <c r="C41" s="4">
-        <f>SUM(C4:C39)</f>
-        <v/>
-      </c>
-      <c r="D41" s="4">
-        <f>SUM(D4:D39)</f>
-        <v/>
-      </c>
+        <f>SUM(B43:B48)</f>
+        <v/>
+      </c>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
       <c r="E41" s="10">
         <f>SUM(E4:E39)</f>
         <v/>

</xml_diff>

<commit_message>
Fix wrong July 6 review data from Jre.xlsx
</commit_message>
<xml_diff>
--- a/data/reviews.xlsx
+++ b/data/reviews.xlsx
@@ -1671,7 +1671,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>21</v>
@@ -1781,7 +1781,7 @@
         <v>4</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>8</v>
@@ -1891,7 +1891,7 @@
         <v>7</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>5</v>
@@ -2001,7 +2001,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>5</v>
@@ -2111,7 +2111,7 @@
         <v>2</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>2</v>
@@ -2221,7 +2221,7 @@
         <v>4</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>5</v>
@@ -2331,7 +2331,7 @@
         <v>9</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>12</v>
@@ -2441,7 +2441,7 @@
         <v>4</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>3</v>
@@ -2551,7 +2551,7 @@
         <v>7</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>4</v>
@@ -2661,7 +2661,7 @@
         <v>4</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>4</v>
@@ -2772,7 +2772,7 @@
         <v>8</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>16</v>
@@ -2882,7 +2882,7 @@
         <v>5</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>7</v>
@@ -2992,7 +2992,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>14</v>
@@ -3102,7 +3102,7 @@
         <v>2</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>0</v>
@@ -3212,7 +3212,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>7</v>
@@ -3322,7 +3322,7 @@
         <v>1</v>
       </c>
       <c r="J19" s="18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>1</v>
@@ -3432,7 +3432,7 @@
         <v>2</v>
       </c>
       <c r="J20" s="18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>4</v>
@@ -3542,7 +3542,7 @@
         <v>10</v>
       </c>
       <c r="J21" s="18" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>5</v>
@@ -3652,7 +3652,7 @@
         <v>11</v>
       </c>
       <c r="J22" s="18" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>8</v>
@@ -3762,7 +3762,7 @@
         <v>3</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>8</v>
@@ -3872,7 +3872,7 @@
         <v>7</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>3</v>
@@ -3982,7 +3982,7 @@
         <v>1</v>
       </c>
       <c r="J25" s="18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>3</v>
@@ -4202,7 +4202,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="18" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>3</v>
@@ -4312,7 +4312,7 @@
         <v>3</v>
       </c>
       <c r="J28" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K28" s="3" t="n">
         <v>2</v>
@@ -4422,7 +4422,7 @@
         <v>16</v>
       </c>
       <c r="J29" s="18" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="K29" s="3" t="n">
         <v>4</v>
@@ -4532,7 +4532,7 @@
         <v>6</v>
       </c>
       <c r="J30" s="18" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>7</v>
@@ -4642,7 +4642,7 @@
         <v>6</v>
       </c>
       <c r="J31" s="18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K31" s="3" t="n">
         <v>9</v>
@@ -4752,7 +4752,7 @@
         <v>2</v>
       </c>
       <c r="J32" s="18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K32" s="3" t="n">
         <v>1</v>
@@ -4862,7 +4862,7 @@
         <v>4</v>
       </c>
       <c r="J33" s="18" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K33" s="3" t="n">
         <v>4</v>
@@ -4972,7 +4972,7 @@
         <v>6</v>
       </c>
       <c r="J34" s="18" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="K34" s="3" t="n">
         <v>1</v>
@@ -5192,7 +5192,7 @@
         <v>5</v>
       </c>
       <c r="J36" s="18" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K36" s="3" t="n">
         <v>9</v>
@@ -5302,7 +5302,7 @@
         <v>3</v>
       </c>
       <c r="J37" s="18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>6</v>
@@ -5412,7 +5412,7 @@
         <v>4</v>
       </c>
       <c r="J38" s="18" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K38" s="3" t="n">
         <v>5</v>
@@ -5696,7 +5696,7 @@
         <v>19</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="K4" s="12" t="inlineStr">
         <is>
@@ -5727,7 +5727,7 @@
         <v>25</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
@@ -5756,7 +5756,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v>21</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K7" s="13" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         <v>44</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
@@ -5843,7 +5843,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
@@ -5872,7 +5872,7 @@
         <v>4</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
@@ -5901,7 +5901,7 @@
         <v>2</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
@@ -5930,7 +5930,7 @@
         <v>2</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
         <v>4</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
         <v>17</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
@@ -6017,7 +6017,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         <v>12</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
@@ -6075,7 +6075,7 @@
         <v>4</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
@@ -6104,7 +6104,7 @@
         <v>4</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
@@ -6133,7 +6133,7 @@
         <v>2</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
@@ -6162,7 +6162,7 @@
         <v>4</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         <v>4</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
@@ -6220,7 +6220,7 @@
         <v>6</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K22" s="13" t="inlineStr">
         <is>
@@ -6249,7 +6249,7 @@
         <v>9</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K23" s="13" t="inlineStr">
         <is>
@@ -6278,7 +6278,7 @@
         <v>7</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K24" s="13" t="inlineStr">
         <is>
@@ -6307,7 +6307,7 @@
         <v>5</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K25" s="13" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>12</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K26" s="13" t="inlineStr">
         <is>
@@ -6365,7 +6365,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K27" s="13" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>4</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K28" s="13" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
         <v>8</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K29" s="13" t="inlineStr">
         <is>
@@ -6452,7 +6452,7 @@
         <v>4</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
@@ -6481,7 +6481,7 @@
         <v>2</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
@@ -6510,7 +6510,7 @@
         <v>8</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
@@ -6539,7 +6539,7 @@
         <v>3</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K33" s="13" t="inlineStr">
         <is>
@@ -6568,7 +6568,7 @@
         <v>8</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
@@ -6597,7 +6597,7 @@
         <v>4</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K35" s="13" t="inlineStr">
         <is>
@@ -6626,7 +6626,7 @@
         <v>12</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" s="13" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         <v>2</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K37" s="13" t="inlineStr">
         <is>
@@ -6684,7 +6684,7 @@
         <v>4</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" s="13" t="inlineStr">
         <is>
@@ -6713,7 +6713,7 @@
         <v>1</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K39" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix July 7 data: replace wrong values with correct data from Jre.xlsx
</commit_message>
<xml_diff>
--- a/data/reviews.xlsx
+++ b/data/reviews.xlsx
@@ -5635,7 +5635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:L50"/>
+  <dimension ref="A2:M50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col width="17.25" customWidth="1" min="1" max="1"/>
@@ -5646,7 +5646,13 @@
     <col width="16.25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="2" ht="1" customHeight="1"/>
+    <row r="2" ht="1" customHeight="1">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="41" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -5708,6 +5714,9 @@
           <t>TARGET</t>
         </is>
       </c>
+      <c r="M4" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -5737,6 +5746,9 @@
       <c r="L5" s="13" t="n">
         <v>25</v>
       </c>
+      <c r="M5" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -5766,6 +5778,9 @@
       <c r="L6" s="13" t="n">
         <v>25</v>
       </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -5795,6 +5810,9 @@
       <c r="L7" s="13" t="n">
         <v>20</v>
       </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -5824,6 +5842,9 @@
       <c r="L8" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="M8" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -5853,6 +5874,9 @@
       <c r="L9" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -5882,6 +5906,9 @@
       <c r="L10" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -5911,6 +5938,9 @@
       <c r="L11" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="M11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -5940,6 +5970,9 @@
       <c r="L12" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -5969,6 +6002,9 @@
       <c r="L13" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -5998,6 +6034,9 @@
       <c r="L14" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="M14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -6027,6 +6066,9 @@
       <c r="L15" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6056,6 +6098,9 @@
       <c r="L16" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="M16" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -6085,6 +6130,9 @@
       <c r="L17" s="13" t="n">
         <v>10</v>
       </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -6114,6 +6162,9 @@
       <c r="L18" s="13" t="n">
         <v>7</v>
       </c>
+      <c r="M18" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -6143,6 +6194,9 @@
       <c r="L19" s="13" t="n">
         <v>7</v>
       </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -6172,6 +6226,9 @@
       <c r="L20" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M20" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -6201,6 +6258,9 @@
       <c r="L21" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -6230,6 +6290,9 @@
       <c r="L22" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -6259,6 +6322,9 @@
       <c r="L23" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M23" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -6288,6 +6354,9 @@
       <c r="L24" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -6317,6 +6386,9 @@
       <c r="L25" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -6346,6 +6418,9 @@
       <c r="L26" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -6375,6 +6450,9 @@
       <c r="L27" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M27" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -6404,6 +6482,9 @@
       <c r="L28" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -6433,6 +6514,9 @@
       <c r="L29" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -6462,6 +6546,9 @@
       <c r="L30" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -6491,6 +6578,9 @@
       <c r="L31" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M31" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -6520,6 +6610,9 @@
       <c r="L32" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M32" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -6549,6 +6642,9 @@
       <c r="L33" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M33" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -6578,6 +6674,9 @@
       <c r="L34" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M34" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -6607,6 +6706,9 @@
       <c r="L35" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -6636,6 +6738,9 @@
       <c r="L36" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -6665,6 +6770,9 @@
       <c r="L37" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M37" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -6694,6 +6802,9 @@
       <c r="L38" s="13" t="n">
         <v>5</v>
       </c>
+      <c r="M38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -6722,6 +6833,9 @@
       </c>
       <c r="L39" s="13" t="n">
         <v>5</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="4" customHeight="1">

</xml_diff>

<commit_message>
Fix July 26 review data from Excel (179->201)
</commit_message>
<xml_diff>
--- a/data/reviews.xlsx
+++ b/data/reviews.xlsx
@@ -1458,7 +1458,7 @@
         </is>
       </c>
       <c r="C4" s="18" t="n">
-        <v>7352</v>
+        <v>7366</v>
       </c>
       <c r="D4" s="3">
         <f>SUM(E4:AH4)</f>
@@ -1537,7 +1537,9 @@
       <c r="AC4" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="AD4" s="21" t="n"/>
+      <c r="AD4" s="21" t="n">
+        <v>23</v>
+      </c>
       <c r="AE4" s="3" t="n"/>
       <c r="AF4" s="3" t="n"/>
       <c r="AG4" s="3" t="n"/>
@@ -1556,7 +1558,7 @@
         </is>
       </c>
       <c r="C5" s="18" t="n">
-        <v>6540</v>
+        <v>6554</v>
       </c>
       <c r="D5" s="3">
         <f>SUM(E5:AH5)</f>
@@ -1635,7 +1637,9 @@
       <c r="AC5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="AD5" s="21" t="n"/>
+      <c r="AD5" s="21" t="n">
+        <v>14</v>
+      </c>
       <c r="AE5" s="3" t="n"/>
       <c r="AF5" s="3" t="n"/>
       <c r="AG5" s="3" t="n"/>
@@ -1654,7 +1658,7 @@
         </is>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="D6" s="3">
         <f>SUM(E6:AH6)</f>
@@ -1733,7 +1737,9 @@
       <c r="AC6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="AD6" s="21" t="n"/>
+      <c r="AD6" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="AE6" s="3" t="n"/>
       <c r="AF6" s="3" t="n"/>
       <c r="AG6" s="3" t="n"/>
@@ -1831,7 +1837,9 @@
       <c r="AC7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="AD7" s="21" t="n"/>
+      <c r="AD7" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="AE7" s="3" t="n"/>
       <c r="AF7" s="3" t="n"/>
       <c r="AG7" s="3" t="n"/>
@@ -1850,7 +1858,7 @@
         </is>
       </c>
       <c r="C8" s="18" t="n">
-        <v>1144</v>
+        <v>1146</v>
       </c>
       <c r="D8" s="3">
         <f>SUM(E8:AH8)</f>
@@ -1929,7 +1937,9 @@
       <c r="AC8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AD8" s="21" t="n"/>
+      <c r="AD8" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE8" s="3" t="n"/>
       <c r="AF8" s="3" t="n"/>
       <c r="AG8" s="3" t="n"/>
@@ -1948,7 +1958,7 @@
         </is>
       </c>
       <c r="C9" s="18" t="n">
-        <v>2067</v>
+        <v>2068</v>
       </c>
       <c r="D9" s="3">
         <f>SUM(E9:AH9)</f>
@@ -2027,7 +2037,9 @@
       <c r="AC9" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="AD9" s="21" t="n"/>
+      <c r="AD9" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="AE9" s="3" t="n"/>
       <c r="AF9" s="3" t="n"/>
       <c r="AG9" s="3" t="n"/>
@@ -2046,7 +2058,7 @@
         </is>
       </c>
       <c r="C10" s="18" t="n">
-        <v>4494</v>
+        <v>4509</v>
       </c>
       <c r="D10" s="3">
         <f>SUM(E10:AH10)</f>
@@ -2125,7 +2137,9 @@
       <c r="AC10" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="AD10" s="21" t="n"/>
+      <c r="AD10" s="21" t="n">
+        <v>23</v>
+      </c>
       <c r="AE10" s="3" t="n"/>
       <c r="AF10" s="3" t="n"/>
       <c r="AG10" s="3" t="n"/>
@@ -2144,7 +2158,7 @@
         </is>
       </c>
       <c r="C11" s="18" t="n">
-        <v>1215</v>
+        <v>1219</v>
       </c>
       <c r="D11" s="3">
         <f>SUM(E11:AH11)</f>
@@ -2223,7 +2237,9 @@
       <c r="AC11" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="AD11" s="21" t="n"/>
+      <c r="AD11" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="AE11" s="3" t="n"/>
       <c r="AF11" s="3" t="n"/>
       <c r="AG11" s="3" t="n"/>
@@ -2242,7 +2258,7 @@
         </is>
       </c>
       <c r="C12" s="18" t="n">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="D12" s="3">
         <f>SUM(E12:AH12)</f>
@@ -2321,7 +2337,9 @@
       <c r="AC12" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="AD12" s="21" t="n"/>
+      <c r="AD12" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="AE12" s="3" t="n"/>
       <c r="AF12" s="3" t="n"/>
       <c r="AG12" s="3" t="n"/>
@@ -2340,7 +2358,7 @@
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="D13" s="3">
         <f>SUM(E13:AH13)</f>
@@ -2419,7 +2437,9 @@
       <c r="AC13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AD13" s="21" t="n"/>
+      <c r="AD13" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE13" s="3" t="n"/>
       <c r="AF13" s="3" t="n"/>
       <c r="AG13" s="3" t="n"/>
@@ -2438,7 +2458,7 @@
         </is>
       </c>
       <c r="C14" s="18" t="n">
-        <v>3204</v>
+        <v>3218</v>
       </c>
       <c r="D14" s="3">
         <f>SUM(E14:AH14)</f>
@@ -2517,7 +2537,9 @@
       <c r="AC14" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="AD14" s="21" t="n"/>
+      <c r="AD14" s="21" t="n">
+        <v>14</v>
+      </c>
       <c r="AE14" s="3" t="n"/>
       <c r="AF14" s="3" t="n"/>
       <c r="AG14" s="3" t="n"/>
@@ -2536,7 +2558,7 @@
         </is>
       </c>
       <c r="C15" s="18" t="n">
-        <v>1148</v>
+        <v>1150</v>
       </c>
       <c r="D15" s="3">
         <f>SUM(E15:AH15)</f>
@@ -2615,7 +2637,9 @@
       <c r="AC15" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AD15" s="21" t="n"/>
+      <c r="AD15" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE15" s="3" t="n"/>
       <c r="AF15" s="3" t="n"/>
       <c r="AG15" s="3" t="n"/>
@@ -2634,7 +2658,7 @@
         </is>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="D16" s="3">
         <f>SUM(E16:AH16)</f>
@@ -2713,7 +2737,9 @@
       <c r="AC16" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="AD16" s="21" t="n"/>
+      <c r="AD16" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE16" s="3" t="n"/>
       <c r="AF16" s="3" t="n"/>
       <c r="AG16" s="3" t="n"/>
@@ -2732,7 +2758,7 @@
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D17" s="3">
         <f>SUM(E17:AH17)</f>
@@ -2811,7 +2837,9 @@
       <c r="AC17" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AD17" s="21" t="n"/>
+      <c r="AD17" s="21" t="n">
+        <v>0</v>
+      </c>
       <c r="AE17" s="3" t="n"/>
       <c r="AF17" s="3" t="n"/>
       <c r="AG17" s="3" t="n"/>
@@ -2830,7 +2858,7 @@
         </is>
       </c>
       <c r="C18" s="18" t="n">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D18" s="3">
         <f>SUM(E18:AH18)</f>
@@ -2909,7 +2937,9 @@
       <c r="AC18" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="AD18" s="21" t="n"/>
+      <c r="AD18" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE18" s="3" t="n"/>
       <c r="AF18" s="3" t="n"/>
       <c r="AG18" s="3" t="n"/>
@@ -2928,7 +2958,7 @@
         </is>
       </c>
       <c r="C19" s="18" t="n">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D19" s="3">
         <f>SUM(E19:AH19)</f>
@@ -3007,7 +3037,9 @@
       <c r="AC19" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="AD19" s="21" t="n"/>
+      <c r="AD19" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE19" s="3" t="n"/>
       <c r="AF19" s="3" t="n"/>
       <c r="AG19" s="3" t="n"/>
@@ -3026,7 +3058,7 @@
         </is>
       </c>
       <c r="C20" s="18" t="n">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="D20" s="3">
         <f>SUM(E20:AH20)</f>
@@ -3105,7 +3137,9 @@
       <c r="AC20" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="AD20" s="21" t="n"/>
+      <c r="AD20" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE20" s="3" t="n"/>
       <c r="AF20" s="3" t="n"/>
       <c r="AG20" s="3" t="n"/>
@@ -3124,7 +3158,7 @@
         </is>
       </c>
       <c r="C21" s="18" t="n">
-        <v>2641</v>
+        <v>2655</v>
       </c>
       <c r="D21" s="3">
         <f>SUM(E21:AH21)</f>
@@ -3203,7 +3237,9 @@
       <c r="AC21" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="AD21" s="21" t="n"/>
+      <c r="AD21" s="21" t="n">
+        <v>14</v>
+      </c>
       <c r="AE21" s="3" t="n"/>
       <c r="AF21" s="3" t="n"/>
       <c r="AG21" s="3" t="n"/>
@@ -3222,7 +3258,7 @@
         </is>
       </c>
       <c r="C22" s="18" t="n">
-        <v>2535</v>
+        <v>2544</v>
       </c>
       <c r="D22" s="3">
         <f>SUM(E22:AH22)</f>
@@ -3301,7 +3337,9 @@
       <c r="AC22" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="AD22" s="21" t="n"/>
+      <c r="AD22" s="21" t="n">
+        <v>11</v>
+      </c>
       <c r="AE22" s="3" t="n"/>
       <c r="AF22" s="3" t="n"/>
       <c r="AG22" s="3" t="n"/>
@@ -3320,7 +3358,7 @@
         </is>
       </c>
       <c r="C23" s="18" t="n">
-        <v>1197</v>
+        <v>1205</v>
       </c>
       <c r="D23" s="3">
         <f>SUM(E23:AH23)</f>
@@ -3399,7 +3437,9 @@
       <c r="AC23" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="AD23" s="21" t="n"/>
+      <c r="AD23" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="AE23" s="3" t="n"/>
       <c r="AF23" s="3" t="n"/>
       <c r="AG23" s="3" t="n"/>
@@ -3418,7 +3458,7 @@
         </is>
       </c>
       <c r="C24" s="18" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D24" s="3">
         <f>SUM(E24:AH24)</f>
@@ -3497,7 +3537,9 @@
       <c r="AC24" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="AD24" s="21" t="n"/>
+      <c r="AD24" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="AE24" s="3" t="n"/>
       <c r="AF24" s="3" t="n"/>
       <c r="AG24" s="3" t="n"/>
@@ -3516,7 +3558,7 @@
         </is>
       </c>
       <c r="C25" s="18" t="n">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="D25" s="3">
         <f>SUM(E25:AH25)</f>
@@ -3595,7 +3637,9 @@
       <c r="AC25" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AD25" s="21" t="n"/>
+      <c r="AD25" s="21" t="n">
+        <v>5</v>
+      </c>
       <c r="AE25" s="3" t="n"/>
       <c r="AF25" s="3" t="n"/>
       <c r="AG25" s="3" t="n"/>
@@ -3614,7 +3658,7 @@
         </is>
       </c>
       <c r="C26" s="18" t="n">
-        <v>1027</v>
+        <v>1013</v>
       </c>
       <c r="D26" s="3">
         <f>SUM(E26:AH26)</f>
@@ -3693,7 +3737,9 @@
       <c r="AC26" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="AD26" s="21" t="n"/>
+      <c r="AD26" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE26" s="3" t="n"/>
       <c r="AF26" s="3" t="n"/>
       <c r="AG26" s="3" t="n"/>
@@ -3791,7 +3837,9 @@
       <c r="AC27" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="AD27" s="21" t="n"/>
+      <c r="AD27" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="AE27" s="3" t="n"/>
       <c r="AF27" s="3" t="n"/>
       <c r="AG27" s="3" t="n"/>
@@ -3810,7 +3858,7 @@
         </is>
       </c>
       <c r="C28" s="18" t="n">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="D28" s="3">
         <f>SUM(E28:AH28)</f>
@@ -3889,7 +3937,9 @@
       <c r="AC28" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AD28" s="21" t="n"/>
+      <c r="AD28" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="AE28" s="3" t="n"/>
       <c r="AF28" s="3" t="n"/>
       <c r="AG28" s="3" t="n"/>
@@ -3908,7 +3958,7 @@
         </is>
       </c>
       <c r="C29" s="18" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D29" s="3">
         <f>SUM(E29:AH29)</f>
@@ -3955,7 +4005,9 @@
       <c r="AC29" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="AD29" s="21" t="n"/>
+      <c r="AD29" s="21" t="n">
+        <v>6</v>
+      </c>
       <c r="AE29" s="3" t="n"/>
       <c r="AF29" s="3" t="n"/>
       <c r="AG29" s="3" t="n"/>
@@ -3974,7 +4026,7 @@
         </is>
       </c>
       <c r="C30" s="18" t="n">
-        <v>6218</v>
+        <v>6224</v>
       </c>
       <c r="D30" s="3">
         <f>SUM(E30:AH30)</f>
@@ -4053,7 +4105,9 @@
       <c r="AC30" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="AD30" s="21" t="n"/>
+      <c r="AD30" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="AE30" s="3" t="n"/>
       <c r="AF30" s="3" t="n"/>
       <c r="AG30" s="3" t="n"/>
@@ -4151,7 +4205,9 @@
       <c r="AC31" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="AD31" s="21" t="n"/>
+      <c r="AD31" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="AE31" s="3" t="n"/>
       <c r="AF31" s="3" t="n"/>
       <c r="AG31" s="3" t="n"/>
@@ -4170,7 +4226,7 @@
         </is>
       </c>
       <c r="C32" s="18" t="n">
-        <v>2320</v>
+        <v>2322</v>
       </c>
       <c r="D32" s="3">
         <f>SUM(E32:AH32)</f>
@@ -4249,7 +4305,9 @@
       <c r="AC32" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="AD32" s="21" t="n"/>
+      <c r="AD32" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE32" s="3" t="n"/>
       <c r="AF32" s="3" t="n"/>
       <c r="AG32" s="3" t="n"/>
@@ -4268,7 +4326,7 @@
         </is>
       </c>
       <c r="C33" s="18" t="n">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="D33" s="3">
         <f>SUM(E33:AH33)</f>
@@ -4347,7 +4405,9 @@
       <c r="AC33" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="AD33" s="21" t="n"/>
+      <c r="AD33" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE33" s="3" t="n"/>
       <c r="AF33" s="3" t="n"/>
       <c r="AG33" s="3" t="n"/>
@@ -4366,7 +4426,7 @@
         </is>
       </c>
       <c r="C34" s="18" t="n">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D34" s="3">
         <f>SUM(E34:AH34)</f>
@@ -4445,7 +4505,9 @@
       <c r="AC34" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="AD34" s="21" t="n"/>
+      <c r="AD34" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="AE34" s="3" t="n"/>
       <c r="AF34" s="3" t="n"/>
       <c r="AG34" s="3" t="n"/>
@@ -4464,7 +4526,7 @@
         </is>
       </c>
       <c r="C35" s="18" t="n">
-        <v>2108</v>
+        <v>2119</v>
       </c>
       <c r="D35" s="3">
         <f>SUM(E35:AH35)</f>
@@ -4543,7 +4605,9 @@
       <c r="AC35" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="AD35" s="21" t="n"/>
+      <c r="AD35" s="21" t="n">
+        <v>12</v>
+      </c>
       <c r="AE35" s="3" t="n"/>
       <c r="AF35" s="3" t="n"/>
       <c r="AG35" s="3" t="n"/>
@@ -4562,7 +4626,7 @@
         </is>
       </c>
       <c r="C36" s="18" t="n">
-        <v>2169</v>
+        <v>2171</v>
       </c>
       <c r="D36" s="3">
         <f>SUM(E36:AH36)</f>
@@ -4641,7 +4705,9 @@
       <c r="AC36" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="AD36" s="21" t="n"/>
+      <c r="AD36" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE36" s="3" t="n"/>
       <c r="AF36" s="3" t="n"/>
       <c r="AG36" s="3" t="n"/>
@@ -4660,7 +4726,7 @@
         </is>
       </c>
       <c r="C37" s="18" t="n">
-        <v>1759</v>
+        <v>1760</v>
       </c>
       <c r="D37" s="3">
         <f>SUM(E37:AH37)</f>
@@ -4739,7 +4805,9 @@
       <c r="AC37" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AD37" s="21" t="n"/>
+      <c r="AD37" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="AE37" s="3" t="n"/>
       <c r="AF37" s="3" t="n"/>
       <c r="AG37" s="3" t="n"/>
@@ -4758,7 +4826,7 @@
         </is>
       </c>
       <c r="C38" s="18" t="n">
-        <v>2105</v>
+        <v>2113</v>
       </c>
       <c r="D38" s="3">
         <f>SUM(E38:AH38)</f>
@@ -4837,7 +4905,9 @@
       <c r="AC38" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="AD38" s="21" t="n"/>
+      <c r="AD38" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="AE38" s="3" t="n"/>
       <c r="AF38" s="3" t="n"/>
       <c r="AG38" s="3" t="n"/>
@@ -4856,7 +4926,7 @@
         </is>
       </c>
       <c r="C39" s="18" t="n">
-        <v>1065</v>
+        <v>1071</v>
       </c>
       <c r="D39" s="3">
         <f>SUM(E39:AH39)</f>
@@ -4935,7 +5005,9 @@
       <c r="AC39" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="AD39" s="21" t="n"/>
+      <c r="AD39" s="21" t="n">
+        <v>7</v>
+      </c>
       <c r="AE39" s="3" t="n"/>
       <c r="AF39" s="3" t="n"/>
       <c r="AG39" s="3" t="n"/>
@@ -4954,7 +5026,7 @@
         </is>
       </c>
       <c r="C40" s="18" t="n">
-        <v>1247</v>
+        <v>1249</v>
       </c>
       <c r="D40" s="3">
         <f>SUM(E40:AH40)</f>
@@ -5033,7 +5105,9 @@
       <c r="AC40" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AD40" s="21" t="n"/>
+      <c r="AD40" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="AE40" s="3" t="n"/>
       <c r="AF40" s="3" t="n"/>
       <c r="AG40" s="3" t="n"/>

</xml_diff>

<commit_message>
Add July 30 reviews data from Jre.xlsx (37 branches, 118 total daily reviews)
</commit_message>
<xml_diff>
--- a/data/reviews.xlsx
+++ b/data/reviews.xlsx
@@ -1458,11 +1458,10 @@
         </is>
       </c>
       <c r="C4" s="18" t="n">
-        <v>7366</v>
-      </c>
-      <c r="D4" s="3">
-        <f>SUM(E4:AH4)</f>
-        <v/>
+        <v>7422</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>708</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>16</v>
@@ -1543,7 +1542,9 @@
       <c r="AE4" s="3" t="n"/>
       <c r="AF4" s="3" t="n"/>
       <c r="AG4" s="3" t="n"/>
-      <c r="AH4" s="3" t="n"/>
+      <c r="AH4" s="3" t="n">
+        <v>26</v>
+      </c>
       <c r="AI4" s="24" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -1558,11 +1559,10 @@
         </is>
       </c>
       <c r="C5" s="18" t="n">
-        <v>6554</v>
-      </c>
-      <c r="D5" s="3">
-        <f>SUM(E5:AH5)</f>
-        <v/>
+        <v>6572</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>187</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>6</v>
@@ -1643,7 +1643,9 @@
       <c r="AE5" s="3" t="n"/>
       <c r="AF5" s="3" t="n"/>
       <c r="AG5" s="3" t="n"/>
-      <c r="AH5" s="3" t="n"/>
+      <c r="AH5" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AI5" s="24" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -1658,11 +1660,10 @@
         </is>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1327</v>
-      </c>
-      <c r="D6" s="3">
-        <f>SUM(E6:AH6)</f>
-        <v/>
+        <v>1337</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>104</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>6</v>
@@ -1743,7 +1744,9 @@
       <c r="AE6" s="3" t="n"/>
       <c r="AF6" s="3" t="n"/>
       <c r="AG6" s="3" t="n"/>
-      <c r="AH6" s="3" t="n"/>
+      <c r="AH6" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="AI6" s="24" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -1758,11 +1761,10 @@
         </is>
       </c>
       <c r="C7" s="18" t="n">
-        <v>430</v>
-      </c>
-      <c r="D7" s="3">
-        <f>SUM(E7:AH7)</f>
-        <v/>
+        <v>434</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>62</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>1</v>
@@ -1843,7 +1845,9 @@
       <c r="AE7" s="3" t="n"/>
       <c r="AF7" s="3" t="n"/>
       <c r="AG7" s="3" t="n"/>
-      <c r="AH7" s="3" t="n"/>
+      <c r="AH7" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI7" s="24" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -1858,11 +1862,10 @@
         </is>
       </c>
       <c r="C8" s="18" t="n">
-        <v>1146</v>
-      </c>
-      <c r="D8" s="3">
-        <f>SUM(E8:AH8)</f>
-        <v/>
+        <v>1148</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>67</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>2</v>
@@ -1943,7 +1946,9 @@
       <c r="AE8" s="3" t="n"/>
       <c r="AF8" s="3" t="n"/>
       <c r="AG8" s="3" t="n"/>
-      <c r="AH8" s="3" t="n"/>
+      <c r="AH8" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI8" s="24" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -1958,11 +1963,10 @@
         </is>
       </c>
       <c r="C9" s="18" t="n">
-        <v>2068</v>
-      </c>
-      <c r="D9" s="3">
-        <f>SUM(E9:AH9)</f>
-        <v/>
+        <v>2076</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>64</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>1</v>
@@ -2043,7 +2047,9 @@
       <c r="AE9" s="3" t="n"/>
       <c r="AF9" s="3" t="n"/>
       <c r="AG9" s="3" t="n"/>
-      <c r="AH9" s="3" t="n"/>
+      <c r="AH9" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI9" s="24" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -2058,11 +2064,10 @@
         </is>
       </c>
       <c r="C10" s="18" t="n">
-        <v>4509</v>
-      </c>
-      <c r="D10" s="3">
-        <f>SUM(E10:AH10)</f>
-        <v/>
+        <v>4502</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>427</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>6</v>
@@ -2143,7 +2148,9 @@
       <c r="AE10" s="3" t="n"/>
       <c r="AF10" s="3" t="n"/>
       <c r="AG10" s="3" t="n"/>
-      <c r="AH10" s="3" t="n"/>
+      <c r="AH10" s="3" t="n">
+        <v>9</v>
+      </c>
       <c r="AI10" s="24" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
@@ -2158,11 +2165,10 @@
         </is>
       </c>
       <c r="C11" s="18" t="n">
-        <v>1219</v>
-      </c>
-      <c r="D11" s="3">
-        <f>SUM(E11:AH11)</f>
-        <v/>
+        <v>1228</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>82</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>1</v>
@@ -2243,7 +2249,9 @@
       <c r="AE11" s="3" t="n"/>
       <c r="AF11" s="3" t="n"/>
       <c r="AG11" s="3" t="n"/>
-      <c r="AH11" s="3" t="n"/>
+      <c r="AH11" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI11" s="24" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -2258,11 +2266,10 @@
         </is>
       </c>
       <c r="C12" s="18" t="n">
-        <v>998</v>
-      </c>
-      <c r="D12" s="3">
-        <f>SUM(E12:AH12)</f>
-        <v/>
+        <v>1000</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>119</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>2</v>
@@ -2343,7 +2350,9 @@
       <c r="AE12" s="3" t="n"/>
       <c r="AF12" s="3" t="n"/>
       <c r="AG12" s="3" t="n"/>
-      <c r="AH12" s="3" t="n"/>
+      <c r="AH12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AI12" s="24" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
@@ -2358,11 +2367,10 @@
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>744</v>
-      </c>
-      <c r="D13" s="3">
-        <f>SUM(E13:AH13)</f>
-        <v/>
+        <v>755</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>59</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1</v>
@@ -2443,7 +2451,9 @@
       <c r="AE13" s="3" t="n"/>
       <c r="AF13" s="3" t="n"/>
       <c r="AG13" s="3" t="n"/>
-      <c r="AH13" s="3" t="n"/>
+      <c r="AH13" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="AI13" s="24" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
@@ -2458,11 +2468,10 @@
         </is>
       </c>
       <c r="C14" s="18" t="n">
-        <v>3218</v>
-      </c>
-      <c r="D14" s="3">
-        <f>SUM(E14:AH14)</f>
-        <v/>
+        <v>3240</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>234</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>5</v>
@@ -2543,7 +2552,9 @@
       <c r="AE14" s="3" t="n"/>
       <c r="AF14" s="3" t="n"/>
       <c r="AG14" s="3" t="n"/>
-      <c r="AH14" s="3" t="n"/>
+      <c r="AH14" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AI14" s="24" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -2558,11 +2569,10 @@
         </is>
       </c>
       <c r="C15" s="18" t="n">
-        <v>1150</v>
-      </c>
-      <c r="D15" s="3">
-        <f>SUM(E15:AH15)</f>
-        <v/>
+        <v>1156</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>42</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>1</v>
@@ -2643,7 +2653,9 @@
       <c r="AE15" s="3" t="n"/>
       <c r="AF15" s="3" t="n"/>
       <c r="AG15" s="3" t="n"/>
-      <c r="AH15" s="3" t="n"/>
+      <c r="AH15" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI15" s="24" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -2658,11 +2670,10 @@
         </is>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1175</v>
-      </c>
-      <c r="D16" s="3">
-        <f>SUM(E16:AH16)</f>
-        <v/>
+        <v>1132</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>69</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>1</v>
@@ -2743,7 +2754,9 @@
       <c r="AE16" s="3" t="n"/>
       <c r="AF16" s="3" t="n"/>
       <c r="AG16" s="3" t="n"/>
-      <c r="AH16" s="3" t="n"/>
+      <c r="AH16" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI16" s="24" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -2760,9 +2773,8 @@
       <c r="C17" s="18" t="n">
         <v>313</v>
       </c>
-      <c r="D17" s="3">
-        <f>SUM(E17:AH17)</f>
-        <v/>
+      <c r="D17" s="3" t="n">
+        <v>41</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>2</v>
@@ -2843,7 +2855,9 @@
       <c r="AE17" s="3" t="n"/>
       <c r="AF17" s="3" t="n"/>
       <c r="AG17" s="3" t="n"/>
-      <c r="AH17" s="3" t="n"/>
+      <c r="AH17" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI17" s="24" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -2858,11 +2872,10 @@
         </is>
       </c>
       <c r="C18" s="18" t="n">
-        <v>455</v>
-      </c>
-      <c r="D18" s="3">
-        <f>SUM(E18:AH18)</f>
-        <v/>
+        <v>457</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>33</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>1</v>
@@ -2943,7 +2956,9 @@
       <c r="AE18" s="3" t="n"/>
       <c r="AF18" s="3" t="n"/>
       <c r="AG18" s="3" t="n"/>
-      <c r="AH18" s="3" t="n"/>
+      <c r="AH18" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI18" s="24" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -2958,11 +2973,10 @@
         </is>
       </c>
       <c r="C19" s="18" t="n">
-        <v>405</v>
-      </c>
-      <c r="D19" s="3">
-        <f>SUM(E19:AH19)</f>
-        <v/>
+        <v>412</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>76</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>3</v>
@@ -3043,7 +3057,9 @@
       <c r="AE19" s="3" t="n"/>
       <c r="AF19" s="3" t="n"/>
       <c r="AG19" s="3" t="n"/>
-      <c r="AH19" s="3" t="n"/>
+      <c r="AH19" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="AI19" s="24" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -3058,11 +3074,10 @@
         </is>
       </c>
       <c r="C20" s="18" t="n">
-        <v>815</v>
-      </c>
-      <c r="D20" s="3">
-        <f>SUM(E20:AH20)</f>
-        <v/>
+        <v>824</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>100</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>1</v>
@@ -3143,7 +3158,9 @@
       <c r="AE20" s="3" t="n"/>
       <c r="AF20" s="3" t="n"/>
       <c r="AG20" s="3" t="n"/>
-      <c r="AH20" s="3" t="n"/>
+      <c r="AH20" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI20" s="24" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -3158,11 +3175,10 @@
         </is>
       </c>
       <c r="C21" s="18" t="n">
-        <v>2655</v>
-      </c>
-      <c r="D21" s="3">
-        <f>SUM(E21:AH21)</f>
-        <v/>
+        <v>2694</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>239</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>3</v>
@@ -3243,7 +3259,9 @@
       <c r="AE21" s="3" t="n"/>
       <c r="AF21" s="3" t="n"/>
       <c r="AG21" s="3" t="n"/>
-      <c r="AH21" s="3" t="n"/>
+      <c r="AH21" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="AI21" s="24" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -3258,11 +3276,10 @@
         </is>
       </c>
       <c r="C22" s="18" t="n">
-        <v>2544</v>
-      </c>
-      <c r="D22" s="3">
-        <f>SUM(E22:AH22)</f>
-        <v/>
+        <v>2559</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>239</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>4</v>
@@ -3343,7 +3360,9 @@
       <c r="AE22" s="3" t="n"/>
       <c r="AF22" s="3" t="n"/>
       <c r="AG22" s="3" t="n"/>
-      <c r="AH22" s="3" t="n"/>
+      <c r="AH22" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI22" s="24" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -3358,11 +3377,10 @@
         </is>
       </c>
       <c r="C23" s="18" t="n">
-        <v>1205</v>
-      </c>
-      <c r="D23" s="3">
-        <f>SUM(E23:AH23)</f>
-        <v/>
+        <v>1220</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>119</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>5</v>
@@ -3443,7 +3461,9 @@
       <c r="AE23" s="3" t="n"/>
       <c r="AF23" s="3" t="n"/>
       <c r="AG23" s="3" t="n"/>
-      <c r="AH23" s="3" t="n"/>
+      <c r="AH23" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AI23" s="24" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -3458,11 +3478,10 @@
         </is>
       </c>
       <c r="C24" s="18" t="n">
-        <v>707</v>
-      </c>
-      <c r="D24" s="3">
-        <f>SUM(E24:AH24)</f>
-        <v/>
+        <v>716</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>64</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>2</v>
@@ -3543,7 +3562,9 @@
       <c r="AE24" s="3" t="n"/>
       <c r="AF24" s="3" t="n"/>
       <c r="AG24" s="3" t="n"/>
-      <c r="AH24" s="3" t="n"/>
+      <c r="AH24" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI24" s="24" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -3558,11 +3579,10 @@
         </is>
       </c>
       <c r="C25" s="18" t="n">
-        <v>670</v>
-      </c>
-      <c r="D25" s="3">
-        <f>SUM(E25:AH25)</f>
-        <v/>
+        <v>683</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>70</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>3</v>
@@ -3643,7 +3663,9 @@
       <c r="AE25" s="3" t="n"/>
       <c r="AF25" s="3" t="n"/>
       <c r="AG25" s="3" t="n"/>
-      <c r="AH25" s="3" t="n"/>
+      <c r="AH25" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="AI25" s="24" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -3658,11 +3680,10 @@
         </is>
       </c>
       <c r="C26" s="18" t="n">
-        <v>1013</v>
-      </c>
-      <c r="D26" s="3">
-        <f>SUM(E26:AH26)</f>
-        <v/>
+        <v>1020</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>64</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>0</v>
@@ -3743,7 +3764,9 @@
       <c r="AE26" s="3" t="n"/>
       <c r="AF26" s="3" t="n"/>
       <c r="AG26" s="3" t="n"/>
-      <c r="AH26" s="3" t="n"/>
+      <c r="AH26" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI26" s="24" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
@@ -3758,11 +3781,10 @@
         </is>
       </c>
       <c r="C27" s="18" t="n">
-        <v>1065</v>
-      </c>
-      <c r="D27" s="3">
-        <f>SUM(E27:AH27)</f>
-        <v/>
+        <v>1068</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>57</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>1</v>
@@ -3843,7 +3865,9 @@
       <c r="AE27" s="3" t="n"/>
       <c r="AF27" s="3" t="n"/>
       <c r="AG27" s="3" t="n"/>
-      <c r="AH27" s="3" t="n"/>
+      <c r="AH27" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AI27" s="24" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
@@ -3858,11 +3882,10 @@
         </is>
       </c>
       <c r="C28" s="18" t="n">
-        <v>1044</v>
-      </c>
-      <c r="D28" s="3">
-        <f>SUM(E28:AH28)</f>
-        <v/>
+        <v>1050</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>115</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>4</v>
@@ -3943,7 +3966,9 @@
       <c r="AE28" s="3" t="n"/>
       <c r="AF28" s="3" t="n"/>
       <c r="AG28" s="3" t="n"/>
-      <c r="AH28" s="3" t="n"/>
+      <c r="AH28" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI28" s="24" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
@@ -3960,9 +3985,8 @@
       <c r="C29" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="D29" s="3">
-        <f>SUM(E29:AH29)</f>
-        <v/>
+      <c r="D29" s="3" t="n">
+        <v>23</v>
       </c>
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
@@ -4011,7 +4035,9 @@
       <c r="AE29" s="3" t="n"/>
       <c r="AF29" s="3" t="n"/>
       <c r="AG29" s="3" t="n"/>
-      <c r="AH29" s="3" t="n"/>
+      <c r="AH29" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AI29" s="24" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -4026,11 +4052,10 @@
         </is>
       </c>
       <c r="C30" s="18" t="n">
-        <v>6224</v>
-      </c>
-      <c r="D30" s="3">
-        <f>SUM(E30:AH30)</f>
-        <v/>
+        <v>6225</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>151</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>9</v>
@@ -4111,7 +4136,9 @@
       <c r="AE30" s="3" t="n"/>
       <c r="AF30" s="3" t="n"/>
       <c r="AG30" s="3" t="n"/>
-      <c r="AH30" s="3" t="n"/>
+      <c r="AH30" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI30" s="24" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -4126,11 +4153,10 @@
         </is>
       </c>
       <c r="C31" s="18" t="n">
-        <v>4048</v>
-      </c>
-      <c r="D31" s="3">
-        <f>SUM(E31:AH31)</f>
-        <v/>
+        <v>4049</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>247</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>12</v>
@@ -4211,7 +4237,9 @@
       <c r="AE31" s="3" t="n"/>
       <c r="AF31" s="3" t="n"/>
       <c r="AG31" s="3" t="n"/>
-      <c r="AH31" s="3" t="n"/>
+      <c r="AH31" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI31" s="24" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -4226,11 +4254,10 @@
         </is>
       </c>
       <c r="C32" s="18" t="n">
-        <v>2322</v>
-      </c>
-      <c r="D32" s="3">
-        <f>SUM(E32:AH32)</f>
-        <v/>
+        <v>2342</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>96</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>2</v>
@@ -4311,7 +4338,9 @@
       <c r="AE32" s="3" t="n"/>
       <c r="AF32" s="3" t="n"/>
       <c r="AG32" s="3" t="n"/>
-      <c r="AH32" s="3" t="n"/>
+      <c r="AH32" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AI32" s="24" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
@@ -4326,11 +4355,10 @@
         </is>
       </c>
       <c r="C33" s="18" t="n">
-        <v>1037</v>
-      </c>
-      <c r="D33" s="3">
-        <f>SUM(E33:AH33)</f>
-        <v/>
+        <v>1039</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>67</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>2</v>
@@ -4411,7 +4439,9 @@
       <c r="AE33" s="3" t="n"/>
       <c r="AF33" s="3" t="n"/>
       <c r="AG33" s="3" t="n"/>
-      <c r="AH33" s="3" t="n"/>
+      <c r="AH33" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI33" s="24" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -4426,11 +4456,10 @@
         </is>
       </c>
       <c r="C34" s="18" t="n">
-        <v>759</v>
-      </c>
-      <c r="D34" s="3">
-        <f>SUM(E34:AH34)</f>
-        <v/>
+        <v>768</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>59</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>0</v>
@@ -4511,7 +4540,9 @@
       <c r="AE34" s="3" t="n"/>
       <c r="AF34" s="3" t="n"/>
       <c r="AG34" s="3" t="n"/>
-      <c r="AH34" s="3" t="n"/>
+      <c r="AH34" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="AI34" s="24" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
@@ -4526,11 +4557,10 @@
         </is>
       </c>
       <c r="C35" s="18" t="n">
-        <v>2119</v>
-      </c>
-      <c r="D35" s="3">
-        <f>SUM(E35:AH35)</f>
-        <v/>
+        <v>2130</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>134</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>7</v>
@@ -4611,7 +4641,9 @@
       <c r="AE35" s="3" t="n"/>
       <c r="AF35" s="3" t="n"/>
       <c r="AG35" s="3" t="n"/>
-      <c r="AH35" s="3" t="n"/>
+      <c r="AH35" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="AI35" s="24" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
@@ -4626,11 +4658,10 @@
         </is>
       </c>
       <c r="C36" s="18" t="n">
-        <v>2171</v>
-      </c>
-      <c r="D36" s="3">
-        <f>SUM(E36:AH36)</f>
-        <v/>
+        <v>2175</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>48</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>1</v>
@@ -4711,7 +4742,9 @@
       <c r="AE36" s="3" t="n"/>
       <c r="AF36" s="3" t="n"/>
       <c r="AG36" s="3" t="n"/>
-      <c r="AH36" s="3" t="n"/>
+      <c r="AH36" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI36" s="24" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
@@ -4726,11 +4759,10 @@
         </is>
       </c>
       <c r="C37" s="18" t="n">
-        <v>1760</v>
-      </c>
-      <c r="D37" s="3">
-        <f>SUM(E37:AH37)</f>
-        <v/>
+        <v>1768</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>97</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>3</v>
@@ -4811,7 +4843,9 @@
       <c r="AE37" s="3" t="n"/>
       <c r="AF37" s="3" t="n"/>
       <c r="AG37" s="3" t="n"/>
-      <c r="AH37" s="3" t="n"/>
+      <c r="AH37" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="AI37" s="24" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
@@ -4826,11 +4860,10 @@
         </is>
       </c>
       <c r="C38" s="18" t="n">
-        <v>2113</v>
-      </c>
-      <c r="D38" s="3">
-        <f>SUM(E38:AH38)</f>
-        <v/>
+        <v>2127</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>111</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>2</v>
@@ -4911,7 +4944,9 @@
       <c r="AE38" s="3" t="n"/>
       <c r="AF38" s="3" t="n"/>
       <c r="AG38" s="3" t="n"/>
-      <c r="AH38" s="3" t="n"/>
+      <c r="AH38" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="AI38" s="24" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -4926,11 +4961,10 @@
         </is>
       </c>
       <c r="C39" s="18" t="n">
-        <v>1071</v>
-      </c>
-      <c r="D39" s="3">
-        <f>SUM(E39:AH39)</f>
-        <v/>
+        <v>985</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>130</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>1</v>
@@ -5011,7 +5045,9 @@
       <c r="AE39" s="3" t="n"/>
       <c r="AF39" s="3" t="n"/>
       <c r="AG39" s="3" t="n"/>
-      <c r="AH39" s="3" t="n"/>
+      <c r="AH39" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="AI39" s="24" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -5026,11 +5062,10 @@
         </is>
       </c>
       <c r="C40" s="18" t="n">
-        <v>1249</v>
-      </c>
-      <c r="D40" s="3">
-        <f>SUM(E40:AH40)</f>
-        <v/>
+        <v>1258</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>57</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>3</v>
@@ -5111,7 +5146,9 @@
       <c r="AE40" s="3" t="n"/>
       <c r="AF40" s="3" t="n"/>
       <c r="AG40" s="3" t="n"/>
-      <c r="AH40" s="3" t="n"/>
+      <c r="AH40" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="AI40" s="24" t="n"/>
     </row>
     <row r="41">
@@ -5204,32 +5241,21 @@
           <t>Tuticorin-1</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+      <c r="B3" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>7352</v>
+        <v>7422</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>587</v>
+        <v>708</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="G3" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A3,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A3,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A3,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A3,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A3,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A3,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K3" s="16" t="inlineStr">
-        <is>
-          <t>Tuticorin-1</t>
-        </is>
-      </c>
-      <c r="L3" s="16" t="n">
-        <v>25</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="G3" s="11" t="n"/>
+      <c r="K3" s="16" t="n"/>
+      <c r="L3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -5237,1179 +5263,789 @@
           <t>Tirunelveli-1</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+      <c r="B4" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>4494</v>
+        <v>4502</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>356</v>
+        <v>427</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="G4" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A4,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A4,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A4,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A4,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A4,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A4,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>Tirunelveli-1</t>
-        </is>
-      </c>
-      <c r="L4" s="16" t="n">
-        <v>25</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="G4" s="11" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="16" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Thenkasi</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Kovilpatti</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>4.7</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3204</v>
+        <v>2694</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>187</v>
+        <v>239</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A5,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A5,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A5,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A5,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A5,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A5,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K5" s="16" t="inlineStr">
-        <is>
-          <t>Thenkasi</t>
-        </is>
-      </c>
-      <c r="L5" s="16" t="n">
-        <v>20</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G5" s="11" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Thenkasi-2</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Monday Market</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2535</v>
+        <v>412</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>198</v>
+        <v>76</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A6,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A6,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A6,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A6,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A6,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A6,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K6" s="16" t="inlineStr">
-        <is>
-          <t>Thenkasi-2</t>
-        </is>
-      </c>
-      <c r="L6" s="16" t="n">
-        <v>15</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G6" s="11" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Ramnad</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>5★</t>
-        </is>
+          <t>Tuticorin-2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>4048</v>
+        <v>6572</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>226</v>
+        <v>187</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="G7" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A7,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A7,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A7,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A7,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A7,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A7,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K7" s="16" t="inlineStr">
-        <is>
-          <t>Kovilpatti</t>
-        </is>
-      </c>
-      <c r="L7" s="16" t="n">
-        <v>15</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Kovilpatti</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Paramakudi</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2105</v>
+        <v>1220</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A8,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A8,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A8,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A8,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A8,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A8,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>Nagercoil</t>
-        </is>
-      </c>
-      <c r="L8" s="16" t="n">
-        <v>15</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G8" s="11" t="n"/>
+      <c r="K8" s="16" t="n"/>
+      <c r="L8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Paramakudi</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Aruppukottai</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>6540</v>
+        <v>2127</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A9,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A9,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A9,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A9,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A9,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A9,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K9" s="16" t="inlineStr">
-        <is>
-          <t>Tuticorin-2</t>
-        </is>
-      </c>
-      <c r="L9" s="16" t="n">
-        <v>15</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G9" s="11" t="n"/>
+      <c r="K9" s="16" t="n"/>
+      <c r="L9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Karungal-1</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>4.7★</t>
-        </is>
+          <t>Thiruchendur-1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>2641</v>
+        <v>1337</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>188</v>
+        <v>104</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A10,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A10,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A10,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A10,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A10,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A10,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K10" s="16" t="inlineStr">
-        <is>
-          <t>Virudhunagar</t>
-        </is>
-      </c>
-      <c r="L10" s="16" t="n">
-        <v>15</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="K10" s="16" t="n"/>
+      <c r="L10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Kayathar-1</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Anjugramam-1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>6218</v>
+        <v>755</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="G11" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A11,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A11,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A11,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A11,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A11,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A11,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K11" s="16" t="inlineStr">
-        <is>
-          <t>Surandai-1</t>
-        </is>
-      </c>
-      <c r="L11" s="16" t="n">
-        <v>10</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G11" s="11" t="n"/>
+      <c r="K11" s="16" t="n"/>
+      <c r="L11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Thiruchendur-1</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Villathikullam</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>994</v>
+        <v>683</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>104</v>
+        <v>70</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A12,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A12,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A12,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A12,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A12,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A12,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K12" s="16" t="inlineStr">
-        <is>
-          <t>Virudhunagar-2</t>
-        </is>
-      </c>
-      <c r="L12" s="16" t="n">
-        <v>10</v>
-      </c>
+      <c r="G12" s="11" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Anjugramam-1</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Rajapalayam</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>453</v>
+        <v>2130</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>29</v>
+        <v>134</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A13,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A13,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A13,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A13,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A13,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A13,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K13" s="16" t="inlineStr">
-        <is>
-          <t>Rajapalayam</t>
-        </is>
-      </c>
-      <c r="L13" s="16" t="n">
-        <v>10</v>
-      </c>
+      <c r="G13" s="11" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Nagercoil</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Ambasamudram-1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>814</v>
+        <v>1000</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G14" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A14,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A14,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A14,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A14,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A14,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A14,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K14" s="16" t="inlineStr">
-        <is>
-          <t>Ambasamudram-1</t>
-        </is>
-      </c>
-      <c r="L14" s="16" t="n">
-        <v>10</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G14" s="11" t="n"/>
+      <c r="K14" s="16" t="n"/>
+      <c r="L14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Sankarankovil-1</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Nagercoil</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1035</v>
+        <v>3240</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>55</v>
+        <v>234</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G15" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A15,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A15,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A15,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A15,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A15,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A15,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K15" s="16" t="inlineStr">
-        <is>
-          <t>Aruppukottai</t>
-        </is>
-      </c>
-      <c r="L15" s="16" t="n">
-        <v>10</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G15" s="11" t="n"/>
+      <c r="K15" s="16" t="n"/>
+      <c r="L15" s="16" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Ramnad-2</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>5★</t>
-        </is>
+          <t>Surandai-1</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>755</v>
+        <v>2342</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G16" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A16,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A16,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A16,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A16,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A16,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A16,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K16" s="16" t="inlineStr">
-        <is>
-          <t>Sayalkudi-1</t>
-        </is>
-      </c>
-      <c r="L16" s="16" t="n">
-        <v>7</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G16" s="11" t="n"/>
+      <c r="K16" s="16" t="n"/>
+      <c r="L16" s="16" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Surandai-1</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Virudhunagar-2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2108</v>
+        <v>1768</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G17" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A17,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A17,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A17,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A17,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A17,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A17,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K17" s="16" t="inlineStr">
-        <is>
-          <t>Ramnad</t>
-        </is>
-      </c>
-      <c r="L17" s="16" t="n">
-        <v>7</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G17" s="11" t="n"/>
+      <c r="K17" s="16" t="n"/>
+      <c r="L17" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Rajapalayam</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Thisayanvilai-1</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G18" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A18,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A18,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A18,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A18,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A18,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A18,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K18" s="16" t="inlineStr">
-        <is>
-          <t>Sivakasi</t>
-        </is>
-      </c>
-      <c r="L18" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G18" s="11" t="n"/>
+      <c r="K18" s="16" t="n"/>
+      <c r="L18" s="16" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Tuticorin-2</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>4.7★</t>
-        </is>
+          <t>Udankudi</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>1173</v>
+        <v>2076</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G19" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A19,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A19,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A19,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A19,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A19,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A19,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K19" s="16" t="inlineStr">
-        <is>
-          <t>Marthandam</t>
-        </is>
-      </c>
-      <c r="L19" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G19" s="11" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="16" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Thisayanvilai-1</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Valliyur-1</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2320</v>
+        <v>1228</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G20" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A20,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A20,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A20,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A20,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A20,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A20,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K20" s="16" t="inlineStr">
-        <is>
-          <t>Thiruchendur-1</t>
-        </is>
-      </c>
-      <c r="L20" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G20" s="11" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Kulasekharam-1</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>5★</t>
-        </is>
+          <t>Karungal-1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1065</v>
+        <v>824</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A21,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A21,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A21,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A21,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A21,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A21,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K21" s="16" t="inlineStr">
-        <is>
-          <t>Sankarankovil-1</t>
-        </is>
-      </c>
-      <c r="L21" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G21" s="11" t="n"/>
+      <c r="K21" s="16" t="n"/>
+      <c r="L21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Aruppukottai -2</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Ramnad</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>1324</v>
+        <v>2559</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>91</v>
+        <v>239</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G22" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A22,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A22,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A22,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A22,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A22,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A22,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K22" s="16" t="inlineStr">
-        <is>
-          <t>Aruppukottai -2</t>
-        </is>
-      </c>
-      <c r="L22" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G22" s="11" t="n"/>
+      <c r="K22" s="16" t="n"/>
+      <c r="L22" s="16" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Eral-2</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Thenkasi</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>1197</v>
+        <v>6225</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>91</v>
+        <v>151</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A23,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A23,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A23,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A23,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A23,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A23,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>Monday Market</t>
-        </is>
-      </c>
-      <c r="L23" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G23" s="11" t="n"/>
+      <c r="K23" s="16" t="n"/>
+      <c r="L23" s="16" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Udankudi</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Thenkasi-2</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>706</v>
+        <v>4049</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>54</v>
+        <v>247</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A24,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A24,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A24,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A24,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A24,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A24,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K24" s="16" t="inlineStr">
-        <is>
-          <t>Puliyankudi-1</t>
-        </is>
-      </c>
-      <c r="L24" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G24" s="11" t="n"/>
+      <c r="K24" s="16" t="n"/>
+      <c r="L24" s="16" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Thuckalay-1</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>5★</t>
-        </is>
+          <t>Sivakasi</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>16</v>
+        <v>1258</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A25,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A25,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A25,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A25,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A25,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A25,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K25" s="16" t="inlineStr">
-        <is>
-          <t>Valliyur-1</t>
-        </is>
-      </c>
-      <c r="L25" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G25" s="11" t="n"/>
+      <c r="K25" s="16" t="n"/>
+      <c r="L25" s="16" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Monday Market</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Eral-2</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>2067</v>
+        <v>1148</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A26,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A26,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A26,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A26,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A26,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A26,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K26" s="16" t="inlineStr">
-        <is>
-          <t>Thuckalay-1</t>
-        </is>
-      </c>
-      <c r="L26" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G26" s="11" t="n"/>
+      <c r="K26" s="16" t="n"/>
+      <c r="L26" s="16" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Sayalkudi-1</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Marthandam</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>4.7</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>1215</v>
+        <v>1156</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A27,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A27,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A27,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A27,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A27,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A27,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K27" s="16" t="inlineStr">
-        <is>
-          <t>Paramakudi</t>
-        </is>
-      </c>
-      <c r="L27" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G27" s="11" t="n"/>
+      <c r="K27" s="16" t="n"/>
+      <c r="L27" s="16" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Sattur-2</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Thuckalay-1</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4.7</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>403</v>
+        <v>1132</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A28,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A28,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A28,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A28,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A28,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A28,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K28" s="16" t="inlineStr">
-        <is>
-          <t>Udankudi</t>
-        </is>
-      </c>
-      <c r="L28" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G28" s="11" t="n"/>
+      <c r="K28" s="16" t="n"/>
+      <c r="L28" s="16" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Puliyankudi-1</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Colachel-1</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>1027</v>
+        <v>313</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A29,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A29,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A29,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A29,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A29,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A29,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K29" s="16" t="inlineStr">
-        <is>
-          <t>Eral-2</t>
-        </is>
-      </c>
-      <c r="L29" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G29" s="11" t="n"/>
+      <c r="K29" s="16" t="n"/>
+      <c r="L29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Virudhunagar-2</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Kulasekharam-1</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1065</v>
+        <v>457</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A30,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A30,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A30,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A30,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A30,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A30,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K30" s="16" t="inlineStr">
-        <is>
-          <t>Colachel-1</t>
-        </is>
-      </c>
-      <c r="L30" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G30" s="11" t="n"/>
+      <c r="K30" s="16" t="n"/>
+      <c r="L30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Aruppukottai</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Sayalkudi-1</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>1144</v>
+        <v>716</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A31,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A31,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A31,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A31,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A31,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A31,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K31" s="16" t="inlineStr">
-        <is>
-          <t>Thisayanvilai-1</t>
-        </is>
-      </c>
-      <c r="L31" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G31" s="11" t="n"/>
+      <c r="K31" s="16" t="n"/>
+      <c r="L31" s="16" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Valliyur-1</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Sattur-2</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>314</v>
+        <v>1020</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A32,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A32,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A32,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A32,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A32,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A32,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K32" s="16" t="inlineStr">
-        <is>
-          <t>Kulasekharam-1</t>
-        </is>
-      </c>
-      <c r="L32" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G32" s="11" t="n"/>
+      <c r="K32" s="16" t="n"/>
+      <c r="L32" s="16" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Ambasamudram-1</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Kayathar-1</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>665</v>
+        <v>1050</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>51</v>
+        <v>115</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A33,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A33,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A33,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A33,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A33,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A33,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K33" s="16" t="inlineStr">
-        <is>
-          <t>Villathikullam</t>
-        </is>
-      </c>
-      <c r="L33" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G33" s="11" t="n"/>
+      <c r="K33" s="16" t="n"/>
+      <c r="L33" s="16" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Colachel-1</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>5★</t>
-        </is>
+          <t>Puliyankudi-1</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G34" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A34,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A34,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A34,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A34,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A34,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A34,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K34" s="16" t="inlineStr">
-        <is>
-          <t>Kayathar-1</t>
-        </is>
-      </c>
-      <c r="L34" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G34" s="11" t="n"/>
+      <c r="K34" s="16" t="n"/>
+      <c r="L34" s="16" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Villathikullam</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Virudhunagar</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>1759</v>
+        <v>2175</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>87</v>
+        <v>48</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G35" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A35,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A35,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A35,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A35,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A35,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A35,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K35" s="16" t="inlineStr">
-        <is>
-          <t>Anjugramam-1</t>
-        </is>
-      </c>
-      <c r="L35" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G35" s="11" t="n"/>
+      <c r="K35" s="16" t="n"/>
+      <c r="L35" s="16" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Sengottai-1</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Aruppukottai -2</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>1247</v>
+        <v>985</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>47</v>
+        <v>130</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A36,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A36,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A36,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A36,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A36,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A36,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K36" s="16" t="inlineStr">
-        <is>
-          <t>Sattur-2</t>
-        </is>
-      </c>
-      <c r="L36" s="16" t="n">
-        <v>5</v>
-      </c>
+      <c r="G36" s="11" t="n"/>
+      <c r="K36" s="16" t="n"/>
+      <c r="L36" s="16" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Virudhunagar</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>4.9★</t>
-        </is>
+          <t>Sankarankovil-1</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>4.9</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>745</v>
+        <v>1068</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A37,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A37,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A37,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A37,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A37,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A37,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K37" s="16" t="inlineStr">
-        <is>
-          <t>Sengottai-1</t>
-        </is>
-      </c>
-      <c r="L37" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G37" s="11" t="n"/>
+      <c r="K37" s="16" t="n"/>
+      <c r="L37" s="16" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Sivakasi</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>4.7★</t>
-        </is>
+          <t>Ramnad-2</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>1148</v>
+        <v>20</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A38,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A38,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A38,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A38,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A38,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A38,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
-      <c r="K38" s="16" t="inlineStr">
-        <is>
-          <t>Karungal-1</t>
-        </is>
-      </c>
-      <c r="L38" s="16" t="n">
-        <v>5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G38" s="11" t="n"/>
+      <c r="K38" s="16" t="n"/>
+      <c r="L38" s="16" t="n"/>
     </row>
     <row r="39" ht="17" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Marthandam</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>4.8★</t>
-        </is>
+          <t>Sengottai-1</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>2169</v>
+        <v>768</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G39" s="11">
-        <f>_xlfn.IFS(ISNUMBER(MATCH(A39,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},0)),"Siva",ISNUMBER(MATCH(A39,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},0)),"John",ISNUMBER(MATCH(A39,{"Thuckalay-1","Nagercoil","Marthandam","Kulasekharam-1","Monday Market","Karungal-1","Colachel-1"},0)),"Jeeva",ISNUMBER(MATCH(A39,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},0)),"Seenivasan",ISNUMBER(MATCH(A39,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Sengottai-1","Rajapalayam"},0)),"Muthuselvam",ISNUMBER(MATCH(A39,{"Virudhunagar","Virudhunagar-2","Aruppukottai -2","Aruppukottai","Sivakasi"},0)),"Venkatesh")</f>
-        <v/>
-      </c>
+      <c r="G39" s="11" t="n"/>
       <c r="K39" s="17" t="n"/>
       <c r="L39" s="17" t="n"/>
     </row>
@@ -6423,129 +6059,49 @@
       <c r="L40" s="15" t="n"/>
     </row>
     <row r="41" ht="18.75" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B41" s="3">
-        <f>VALUE(SUBSTITUTE(B3,"★",""))</f>
-        <v/>
-      </c>
-      <c r="C41" s="4">
-        <f>SUM(C3:C39)</f>
-        <v/>
-      </c>
-      <c r="D41" s="4">
-        <f>SUM(D3:D39)</f>
-        <v/>
-      </c>
-      <c r="E41" s="13">
-        <f>SUM(E3:E39)</f>
-        <v/>
-      </c>
-      <c r="K41" s="15" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="L41" s="15">
-        <f>SUM(L3:L38)</f>
-        <v/>
-      </c>
+      <c r="A41" s="3" t="n"/>
+      <c r="B41" s="3" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="13" t="n"/>
+      <c r="K41" s="15" t="n"/>
+      <c r="L41" s="15" t="n"/>
     </row>
     <row r="42" ht="27" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>Monthly Total</t>
-        </is>
-      </c>
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="6" t="n"/>
     </row>
     <row r="43" ht="17.25" customHeight="1">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>TKS1</t>
-        </is>
-      </c>
-      <c r="B43" s="7">
-        <f>SUM(SUMIF(A3:A39,{"Thenkasi","Thenkasi-2","Surandai-1","Puliyankudi-1","Rajapalayam","Sengottai-1"},D3:D39))</f>
-        <v/>
-      </c>
+      <c r="A43" s="7" t="n"/>
+      <c r="B43" s="7" t="n"/>
     </row>
     <row r="44" ht="17.25" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>Tuticorin</t>
-        </is>
-      </c>
-      <c r="B44" s="7">
-        <f>SUM(SUMIF(A3:A39,{"Tuticorin-1","Tuticorin-2","Thiruchendur-1","Thisayanvilai-1","Eral-2","Udankudi"},D3:D39))</f>
-        <v/>
-      </c>
+      <c r="A44" s="7" t="n"/>
+      <c r="B44" s="7" t="n"/>
     </row>
     <row r="45" ht="17.25" customHeight="1">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>Tirunelveli</t>
-        </is>
-      </c>
-      <c r="B45" s="7">
-        <f>SUM(SUMIF(A3:A39,{"Tirunelveli-1","Valliyur-1","Ambasamudram-1","Anjugramam-1"},D3:D39))</f>
-        <v/>
-      </c>
+      <c r="A45" s="7" t="n"/>
+      <c r="B45" s="7" t="n"/>
     </row>
     <row r="46" ht="17.25" customHeight="1">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>VNR1</t>
-        </is>
-      </c>
-      <c r="B46" s="7">
-        <f>SUM(SUMIF(A3:A39,{"Virudhunagar","Virudhunagar-2","Aruppukottai","Aruppukottai -2","Sivakasi"},D3:D39))</f>
-        <v/>
-      </c>
+      <c r="A46" s="7" t="n"/>
+      <c r="B46" s="7" t="n"/>
     </row>
     <row r="47" ht="17.25" customHeight="1">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>NGR1</t>
-        </is>
-      </c>
-      <c r="B47" s="7">
-        <f>SUM(SUMIF(A3:A39,{"Nagercoil","Marthandam","Thuckalay-1","Colachel-1","Kulasekharam-1","Monday Market","Karungal-1"},D3:D39))</f>
-        <v/>
-      </c>
+      <c r="A47" s="7" t="n"/>
+      <c r="B47" s="7" t="n"/>
     </row>
     <row r="48" ht="17.25" customHeight="1">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>KVT1</t>
-        </is>
-      </c>
-      <c r="B48" s="7">
-        <f>SUM(SUMIF(A3:A39,{"Kovilpatti","Ramnad","Ramnad-2","Paramakudi","Sayalkudi-1","Villathikullam","Sattur-2","Sankarankovil-1","Kayathar-1"},D3:D39))</f>
-        <v/>
-      </c>
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
     </row>
     <row r="49" ht="3" customHeight="1">
       <c r="A49" s="7" t="n"/>
       <c r="B49" s="29" t="n"/>
     </row>
     <row r="50" ht="17.25" customHeight="1">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B50" s="7">
-        <f>SUM(B43:B48)</f>
-        <v/>
-      </c>
+      <c r="A50" s="7" t="n"/>
+      <c r="B50" s="7" t="n"/>
     </row>
     <row r="51" ht="16.5" customHeight="1"/>
   </sheetData>

</xml_diff>